<commit_message>
Enhance eBay listing generation by adding HTML output for each listing and updating README for bulk upload instructions. Refactor .gitignore to include new HTML directory and improve YAML settings for eBay API integration. Update documentation for clarity on usage and project structure.
</commit_message>
<xml_diff>
--- a/data/my_cards.xlsx
+++ b/data/my_cards.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\camauger\OneDrive - Université TÉLUQ\Bureau\sites\lotrtcg.shop\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://teluq-my.sharepoint.com/personal/christian_amauger_teluq_ca/Documents/Bureau/sites/lotrtcg.shop/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60A9B947-A6D8-4196-B1D9-FF8BE1167177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="104" documentId="13_ncr:1_{60A9B947-A6D8-4196-B1D9-FF8BE1167177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{627C1A76-AF0C-4D11-B9B0-A193901A2725}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5502F620-63D6-485D-ACFA-8F5F25F0D7CC}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="104">
   <si>
     <t>Set</t>
   </si>
@@ -278,13 +278,67 @@
   </si>
   <si>
     <t>11.95</t>
+  </si>
+  <si>
+    <t>1R90</t>
+  </si>
+  <si>
+    <t>0P41</t>
+  </si>
+  <si>
+    <t>6R126</t>
+  </si>
+  <si>
+    <t>15C65</t>
+  </si>
+  <si>
+    <t>6C56</t>
+  </si>
+  <si>
+    <t>3R42</t>
+  </si>
+  <si>
+    <t>14R8</t>
+  </si>
+  <si>
+    <t>14R9</t>
+  </si>
+  <si>
+    <t>13R65</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 8R36 </t>
+  </si>
+  <si>
+    <t>8R37</t>
+  </si>
+  <si>
+    <t>9+R32</t>
+  </si>
+  <si>
+    <t>3R13</t>
+  </si>
+  <si>
+    <t>7R1</t>
+  </si>
+  <si>
+    <t>12R17</t>
+  </si>
+  <si>
+    <t>11RF3</t>
+  </si>
+  <si>
+    <t>1R50</t>
+  </si>
+  <si>
+    <t>10R18</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -424,6 +478,12 @@
       <color rgb="FF191919"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1145,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D9C976C-E522-4B3D-926B-45327FDC26DA}">
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G85"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -2471,27 +2531,408 @@
         <v>4</v>
       </c>
     </row>
+    <row r="67" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B67" t="s">
+        <v>86</v>
+      </c>
+      <c r="C67" t="s">
+        <v>7</v>
+      </c>
+      <c r="D67" t="s">
+        <v>8</v>
+      </c>
+      <c r="E67" t="s">
+        <v>9</v>
+      </c>
+      <c r="F67">
+        <v>9</v>
+      </c>
+      <c r="G67">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="68" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B68" t="s">
+        <v>87</v>
+      </c>
+      <c r="C68" t="s">
+        <v>7</v>
+      </c>
+      <c r="D68" t="s">
+        <v>8</v>
+      </c>
+      <c r="E68" t="s">
+        <v>9</v>
+      </c>
+      <c r="F68">
+        <v>3</v>
+      </c>
+      <c r="G68">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B69" t="s">
+        <v>88</v>
+      </c>
+      <c r="C69" t="s">
+        <v>7</v>
+      </c>
+      <c r="D69" t="s">
+        <v>8</v>
+      </c>
+      <c r="E69" t="s">
+        <v>9</v>
+      </c>
+      <c r="F69">
+        <v>3</v>
+      </c>
+      <c r="G69">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B70" t="s">
+        <v>89</v>
+      </c>
+      <c r="C70" t="s">
+        <v>7</v>
+      </c>
+      <c r="D70" t="s">
+        <v>8</v>
+      </c>
+      <c r="E70" t="s">
+        <v>9</v>
+      </c>
+      <c r="F70">
+        <v>1</v>
+      </c>
+      <c r="G70">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="71" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B71" t="s">
+        <v>90</v>
+      </c>
+      <c r="C71" t="s">
+        <v>7</v>
+      </c>
+      <c r="D71" t="s">
+        <v>8</v>
+      </c>
+      <c r="E71" t="s">
+        <v>12</v>
+      </c>
+      <c r="F71">
+        <v>3</v>
+      </c>
+      <c r="G71">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="72" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B72" t="s">
+        <v>91</v>
+      </c>
+      <c r="C72" t="s">
+        <v>7</v>
+      </c>
+      <c r="D72" t="s">
+        <v>8</v>
+      </c>
+      <c r="E72" t="s">
+        <v>9</v>
+      </c>
+      <c r="F72">
+        <v>5</v>
+      </c>
+      <c r="G72">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="73" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B73" t="s">
+        <v>92</v>
+      </c>
+      <c r="C73" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73" t="s">
+        <v>8</v>
+      </c>
+      <c r="E73" t="s">
+        <v>9</v>
+      </c>
+      <c r="F73">
+        <v>7</v>
+      </c>
+      <c r="G73">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="74" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B74" t="s">
+        <v>93</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74" t="s">
+        <v>8</v>
+      </c>
+      <c r="E74" t="s">
+        <v>9</v>
+      </c>
+      <c r="F74">
+        <v>12</v>
+      </c>
+      <c r="G74">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="75" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B75" t="s">
+        <v>94</v>
+      </c>
+      <c r="C75" t="s">
+        <v>7</v>
+      </c>
+      <c r="D75" t="s">
+        <v>8</v>
+      </c>
+      <c r="E75" t="s">
+        <v>9</v>
+      </c>
+      <c r="F75">
+        <v>55</v>
+      </c>
+      <c r="G75">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="76" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B76" t="s">
+        <v>95</v>
+      </c>
+      <c r="C76" t="s">
+        <v>7</v>
+      </c>
+      <c r="D76" t="s">
+        <v>8</v>
+      </c>
+      <c r="E76" t="s">
+        <v>12</v>
+      </c>
+      <c r="F76">
+        <v>65</v>
+      </c>
+      <c r="G76">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B77" t="s">
+        <v>96</v>
+      </c>
+      <c r="C77" t="s">
+        <v>7</v>
+      </c>
+      <c r="D77" t="s">
+        <v>8</v>
+      </c>
+      <c r="E77" t="s">
+        <v>12</v>
+      </c>
+      <c r="F77">
+        <v>30</v>
+      </c>
+      <c r="G77">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B78" t="s">
+        <v>97</v>
+      </c>
+      <c r="C78" t="s">
+        <v>7</v>
+      </c>
+      <c r="D78" t="s">
+        <v>8</v>
+      </c>
+      <c r="E78" t="s">
+        <v>12</v>
+      </c>
+      <c r="F78">
+        <v>25</v>
+      </c>
+      <c r="G78">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="79" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B79" t="s">
+        <v>98</v>
+      </c>
+      <c r="C79" t="s">
+        <v>7</v>
+      </c>
+      <c r="D79" t="s">
+        <v>8</v>
+      </c>
+      <c r="E79" t="s">
+        <v>9</v>
+      </c>
+      <c r="F79">
+        <v>22</v>
+      </c>
+      <c r="G79">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="80" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B80" t="s">
+        <v>99</v>
+      </c>
+      <c r="C80" t="s">
+        <v>7</v>
+      </c>
+      <c r="D80" t="s">
+        <v>8</v>
+      </c>
+      <c r="E80" t="s">
+        <v>9</v>
+      </c>
+      <c r="F80">
+        <v>9</v>
+      </c>
+      <c r="G80">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B81" t="s">
+        <v>100</v>
+      </c>
+      <c r="C81" t="s">
+        <v>7</v>
+      </c>
+      <c r="D81" t="s">
+        <v>8</v>
+      </c>
+      <c r="E81" t="s">
+        <v>12</v>
+      </c>
+      <c r="F81">
+        <v>9</v>
+      </c>
+      <c r="G81">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="82" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B82" t="s">
+        <v>100</v>
+      </c>
+      <c r="C82" t="s">
+        <v>7</v>
+      </c>
+      <c r="D82" t="s">
+        <v>8</v>
+      </c>
+      <c r="E82" t="s">
+        <v>9</v>
+      </c>
+      <c r="F82">
+        <v>5</v>
+      </c>
+      <c r="G82">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B83" t="s">
+        <v>101</v>
+      </c>
+      <c r="C83" t="s">
+        <v>7</v>
+      </c>
+      <c r="D83" t="s">
+        <v>8</v>
+      </c>
+      <c r="E83" t="s">
+        <v>12</v>
+      </c>
+      <c r="F83">
+        <v>9</v>
+      </c>
+      <c r="G83">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="84" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B84" t="s">
+        <v>102</v>
+      </c>
+      <c r="C84" t="s">
+        <v>7</v>
+      </c>
+      <c r="D84" t="s">
+        <v>8</v>
+      </c>
+      <c r="E84" t="s">
+        <v>9</v>
+      </c>
+      <c r="F84">
+        <v>15</v>
+      </c>
+      <c r="G84">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="85" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B85" t="s">
+        <v>103</v>
+      </c>
+      <c r="C85" t="s">
+        <v>7</v>
+      </c>
+      <c r="D85" t="s">
+        <v>8</v>
+      </c>
+      <c r="E85" t="s">
+        <v>9</v>
+      </c>
+      <c r="F85">
+        <v>15</v>
+      </c>
+      <c r="G85">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="19" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="633964cd-1e87-40d0-a301-310797c49dfe" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="633964cd-1e87-40d0-a301-310797c49dfe" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2734,6 +3175,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD0ABDC5-64C7-46E1-B4D8-32E7F6B4A3B4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{89D9FA58-1183-48E6-8E36-E83B101C2F79}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -2746,14 +3195,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="633964cd-1e87-40d0-a301-310797c49dfe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD0ABDC5-64C7-46E1-B4D8-32E7F6B4A3B4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>